<commit_message>
feat: measured the optimal block size of risk-V
</commit_message>
<xml_diff>
--- a/DecompositionLU/docs/version_3.2_statistics.xlsx
+++ b/DecompositionLU/docs/version_3.2_statistics.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Maxim\source\repos\practice\SECOND_COURSE\FOR_ITLAB\ArchBenchs\DecompositionLU\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36476871-5B0C-44C9-99AF-08F53CABC895}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3A3883F-4249-4585-ACBF-20DC4AA82CB9}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-114" yWindow="-114" windowWidth="27602" windowHeight="15027" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-114" yWindow="-114" windowWidth="27602" windowHeight="15027" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Графики" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="32">
   <si>
     <t>Замеры версии 3.2</t>
   </si>
@@ -228,6 +228,12 @@
       <t>кластер risk-V</t>
     </r>
   </si>
+  <si>
+    <t>размер блока:</t>
+  </si>
+  <si>
+    <t>n</t>
+  </si>
 </sst>
 </file>
 
@@ -397,7 +403,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -477,12 +483,38 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="62">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
@@ -532,6 +564,36 @@
     <xf numFmtId="0" fontId="5" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -540,6 +602,33 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -559,63 +648,31 @@
     <xf numFmtId="0" fontId="4" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="3" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -29301,30 +29358,30 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="31" t="s">
+      <c r="A1" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="32"/>
-      <c r="C1" s="32"/>
-      <c r="D1" s="32"/>
-      <c r="E1" s="32"/>
-      <c r="F1" s="32"/>
-      <c r="G1" s="32"/>
-      <c r="H1" s="32"/>
-      <c r="I1" s="32"/>
-      <c r="J1" s="32"/>
-      <c r="K1" s="32"/>
-      <c r="L1" s="32"/>
-      <c r="M1" s="32"/>
-      <c r="N1" s="32"/>
-      <c r="O1" s="50" t="s">
+      <c r="B1" s="43"/>
+      <c r="C1" s="43"/>
+      <c r="D1" s="43"/>
+      <c r="E1" s="43"/>
+      <c r="F1" s="43"/>
+      <c r="G1" s="43"/>
+      <c r="H1" s="43"/>
+      <c r="I1" s="43"/>
+      <c r="J1" s="43"/>
+      <c r="K1" s="43"/>
+      <c r="L1" s="43"/>
+      <c r="M1" s="43"/>
+      <c r="N1" s="43"/>
+      <c r="O1" s="44" t="s">
         <v>1</v>
       </c>
-      <c r="P1" s="51"/>
-      <c r="Q1" s="51"/>
-      <c r="R1" s="51"/>
-      <c r="S1" s="51"/>
-      <c r="T1" s="52"/>
+      <c r="P1" s="45"/>
+      <c r="Q1" s="45"/>
+      <c r="R1" s="45"/>
+      <c r="S1" s="45"/>
+      <c r="T1" s="46"/>
       <c r="U1" s="1"/>
       <c r="V1" s="1"/>
       <c r="W1" s="1"/>
@@ -29336,15 +29393,15 @@
       <c r="AC1" s="1"/>
     </row>
     <row r="2" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="28" t="s">
+      <c r="A2" s="39" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="22" t="s">
+      <c r="B2" s="47" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="23"/>
-      <c r="D2" s="23"/>
-      <c r="E2" s="24"/>
+      <c r="C2" s="48"/>
+      <c r="D2" s="48"/>
+      <c r="E2" s="49"/>
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
       <c r="H2" s="2"/>
@@ -29371,7 +29428,7 @@
       <c r="AC2" s="1"/>
     </row>
     <row r="3" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="28"/>
+      <c r="A3" s="39"/>
       <c r="B3" s="3" t="s">
         <v>4</v>
       </c>
@@ -29410,7 +29467,7 @@
       <c r="AC3" s="1"/>
     </row>
     <row r="4" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="28"/>
+      <c r="A4" s="39"/>
       <c r="B4" s="4">
         <v>1</v>
       </c>
@@ -29449,7 +29506,7 @@
       <c r="AC4" s="1"/>
     </row>
     <row r="5" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="28"/>
+      <c r="A5" s="39"/>
       <c r="B5" s="4">
         <v>2</v>
       </c>
@@ -29488,7 +29545,7 @@
       <c r="AC5" s="1"/>
     </row>
     <row r="6" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="28"/>
+      <c r="A6" s="39"/>
       <c r="B6" s="4">
         <v>4</v>
       </c>
@@ -29527,7 +29584,7 @@
       <c r="AC6" s="1"/>
     </row>
     <row r="7" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="28"/>
+      <c r="A7" s="39"/>
       <c r="B7" s="4">
         <v>6</v>
       </c>
@@ -29566,7 +29623,7 @@
       <c r="AC7" s="1"/>
     </row>
     <row r="8" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="28"/>
+      <c r="A8" s="39"/>
       <c r="B8" s="4">
         <v>8</v>
       </c>
@@ -29605,7 +29662,7 @@
       <c r="AC8" s="1"/>
     </row>
     <row r="9" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="28"/>
+      <c r="A9" s="39"/>
       <c r="B9" s="4">
         <v>10</v>
       </c>
@@ -29644,7 +29701,7 @@
       <c r="AC9" s="1"/>
     </row>
     <row r="10" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="28"/>
+      <c r="A10" s="39"/>
       <c r="B10" s="4">
         <v>12</v>
       </c>
@@ -29683,7 +29740,7 @@
       <c r="AC10" s="1"/>
     </row>
     <row r="11" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="28"/>
+      <c r="A11" s="39"/>
       <c r="B11" s="4">
         <v>16</v>
       </c>
@@ -29722,13 +29779,13 @@
       <c r="AC11" s="1"/>
     </row>
     <row r="12" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="28"/>
-      <c r="B12" s="22" t="s">
+      <c r="A12" s="39"/>
+      <c r="B12" s="47" t="s">
         <v>8</v>
       </c>
-      <c r="C12" s="23"/>
-      <c r="D12" s="23"/>
-      <c r="E12" s="24"/>
+      <c r="C12" s="48"/>
+      <c r="D12" s="48"/>
+      <c r="E12" s="49"/>
       <c r="F12" s="2"/>
       <c r="G12" s="2"/>
       <c r="H12" s="2"/>
@@ -29755,7 +29812,7 @@
       <c r="AC12" s="1"/>
     </row>
     <row r="13" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="28"/>
+      <c r="A13" s="39"/>
       <c r="B13" s="3" t="s">
         <v>4</v>
       </c>
@@ -29794,7 +29851,7 @@
       <c r="AC13" s="1"/>
     </row>
     <row r="14" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="28"/>
+      <c r="A14" s="39"/>
       <c r="B14" s="3">
         <v>1</v>
       </c>
@@ -29836,7 +29893,7 @@
       <c r="AC14" s="1"/>
     </row>
     <row r="15" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="28"/>
+      <c r="A15" s="39"/>
       <c r="B15" s="3">
         <v>2</v>
       </c>
@@ -29878,7 +29935,7 @@
       <c r="AC15" s="1"/>
     </row>
     <row r="16" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="28"/>
+      <c r="A16" s="39"/>
       <c r="B16" s="3">
         <v>4</v>
       </c>
@@ -29920,7 +29977,7 @@
       <c r="AC16" s="1"/>
     </row>
     <row r="17" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="28"/>
+      <c r="A17" s="39"/>
       <c r="B17" s="3">
         <v>6</v>
       </c>
@@ -29962,7 +30019,7 @@
       <c r="AC17" s="1"/>
     </row>
     <row r="18" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="28"/>
+      <c r="A18" s="39"/>
       <c r="B18" s="3">
         <v>8</v>
       </c>
@@ -30004,7 +30061,7 @@
       <c r="AC18" s="1"/>
     </row>
     <row r="19" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="28"/>
+      <c r="A19" s="39"/>
       <c r="B19" s="3">
         <v>10</v>
       </c>
@@ -30046,7 +30103,7 @@
       <c r="AC19" s="1"/>
     </row>
     <row r="20" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="28"/>
+      <c r="A20" s="39"/>
       <c r="B20" s="3">
         <v>12</v>
       </c>
@@ -30088,7 +30145,7 @@
       <c r="AC20" s="1"/>
     </row>
     <row r="21" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="28"/>
+      <c r="A21" s="39"/>
       <c r="B21" s="3">
         <v>16</v>
       </c>
@@ -30130,13 +30187,13 @@
       <c r="AC21" s="1"/>
     </row>
     <row r="22" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="28"/>
-      <c r="B22" s="22" t="s">
+      <c r="A22" s="39"/>
+      <c r="B22" s="47" t="s">
         <v>9</v>
       </c>
-      <c r="C22" s="23"/>
-      <c r="D22" s="23"/>
-      <c r="E22" s="24"/>
+      <c r="C22" s="48"/>
+      <c r="D22" s="48"/>
+      <c r="E22" s="49"/>
       <c r="F22" s="7"/>
       <c r="G22" s="8"/>
       <c r="H22" s="8"/>
@@ -30163,7 +30220,7 @@
       <c r="AC22" s="1"/>
     </row>
     <row r="23" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="28"/>
+      <c r="A23" s="39"/>
       <c r="B23" s="3" t="s">
         <v>4</v>
       </c>
@@ -30202,7 +30259,7 @@
       <c r="AC23" s="1"/>
     </row>
     <row r="24" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="28"/>
+      <c r="A24" s="39"/>
       <c r="B24" s="3">
         <v>1</v>
       </c>
@@ -30244,7 +30301,7 @@
       <c r="AC24" s="1"/>
     </row>
     <row r="25" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="28"/>
+      <c r="A25" s="39"/>
       <c r="B25" s="3">
         <v>2</v>
       </c>
@@ -30286,7 +30343,7 @@
       <c r="AC25" s="1"/>
     </row>
     <row r="26" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="28"/>
+      <c r="A26" s="39"/>
       <c r="B26" s="3">
         <v>4</v>
       </c>
@@ -30328,7 +30385,7 @@
       <c r="AC26" s="1"/>
     </row>
     <row r="27" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="28"/>
+      <c r="A27" s="39"/>
       <c r="B27" s="3">
         <v>6</v>
       </c>
@@ -30370,7 +30427,7 @@
       <c r="AC27" s="1"/>
     </row>
     <row r="28" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="28"/>
+      <c r="A28" s="39"/>
       <c r="B28" s="3">
         <v>8</v>
       </c>
@@ -30412,7 +30469,7 @@
       <c r="AC28" s="1"/>
     </row>
     <row r="29" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="28"/>
+      <c r="A29" s="39"/>
       <c r="B29" s="3">
         <v>10</v>
       </c>
@@ -30454,7 +30511,7 @@
       <c r="AC29" s="1"/>
     </row>
     <row r="30" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="28"/>
+      <c r="A30" s="39"/>
       <c r="B30" s="3">
         <v>12</v>
       </c>
@@ -30496,7 +30553,7 @@
       <c r="AC30" s="1"/>
     </row>
     <row r="31" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="28"/>
+      <c r="A31" s="39"/>
       <c r="B31" s="3">
         <v>16</v>
       </c>
@@ -30538,30 +30595,30 @@
       <c r="AC31" s="1"/>
     </row>
     <row r="32" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="28"/>
+      <c r="A32" s="39"/>
       <c r="B32" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="C32" s="25" t="s">
+      <c r="C32" s="50" t="s">
         <v>11</v>
       </c>
-      <c r="D32" s="26"/>
-      <c r="E32" s="26"/>
-      <c r="F32" s="26"/>
-      <c r="G32" s="26"/>
-      <c r="H32" s="26"/>
-      <c r="I32" s="26"/>
-      <c r="J32" s="26"/>
-      <c r="K32" s="26"/>
-      <c r="L32" s="26"/>
-      <c r="M32" s="26"/>
-      <c r="N32" s="26"/>
-      <c r="O32" s="26"/>
-      <c r="P32" s="26"/>
-      <c r="Q32" s="26"/>
-      <c r="R32" s="26"/>
-      <c r="S32" s="26"/>
-      <c r="T32" s="27"/>
+      <c r="D32" s="51"/>
+      <c r="E32" s="51"/>
+      <c r="F32" s="51"/>
+      <c r="G32" s="51"/>
+      <c r="H32" s="51"/>
+      <c r="I32" s="51"/>
+      <c r="J32" s="51"/>
+      <c r="K32" s="51"/>
+      <c r="L32" s="51"/>
+      <c r="M32" s="51"/>
+      <c r="N32" s="51"/>
+      <c r="O32" s="51"/>
+      <c r="P32" s="51"/>
+      <c r="Q32" s="51"/>
+      <c r="R32" s="51"/>
+      <c r="S32" s="51"/>
+      <c r="T32" s="52"/>
       <c r="U32" s="1"/>
       <c r="V32" s="1"/>
       <c r="W32" s="1"/>
@@ -30573,15 +30630,15 @@
       <c r="AC32" s="1"/>
     </row>
     <row r="33" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="20" t="s">
+      <c r="A33" s="36" t="s">
         <v>12</v>
       </c>
-      <c r="B33" s="29" t="s">
+      <c r="B33" s="38" t="s">
         <v>3</v>
       </c>
-      <c r="C33" s="29"/>
-      <c r="D33" s="29"/>
-      <c r="E33" s="29"/>
+      <c r="C33" s="38"/>
+      <c r="D33" s="38"/>
+      <c r="E33" s="38"/>
       <c r="F33" s="2"/>
       <c r="G33" s="2"/>
       <c r="H33" s="2"/>
@@ -30604,11 +30661,11 @@
       <c r="Y33" s="2"/>
       <c r="Z33" s="2"/>
       <c r="AA33" s="2"/>
-      <c r="AB33" s="33"/>
-      <c r="AC33" s="33"/>
+      <c r="AB33" s="19"/>
+      <c r="AC33" s="19"/>
     </row>
     <row r="34" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="21"/>
+      <c r="A34" s="37"/>
       <c r="B34" s="3" t="s">
         <v>4</v>
       </c>
@@ -30643,11 +30700,11 @@
       <c r="Y34" s="2"/>
       <c r="Z34" s="2"/>
       <c r="AA34" s="2"/>
-      <c r="AB34" s="33"/>
-      <c r="AC34" s="33"/>
+      <c r="AB34" s="19"/>
+      <c r="AC34" s="19"/>
     </row>
     <row r="35" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="21"/>
+      <c r="A35" s="37"/>
       <c r="B35" s="4">
         <v>1</v>
       </c>
@@ -30682,11 +30739,11 @@
       <c r="Y35" s="2"/>
       <c r="Z35" s="2"/>
       <c r="AA35" s="2"/>
-      <c r="AB35" s="33"/>
-      <c r="AC35" s="33"/>
+      <c r="AB35" s="19"/>
+      <c r="AC35" s="19"/>
     </row>
     <row r="36" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="21"/>
+      <c r="A36" s="37"/>
       <c r="B36" s="4">
         <v>2</v>
       </c>
@@ -30721,11 +30778,11 @@
       <c r="Y36" s="2"/>
       <c r="Z36" s="2"/>
       <c r="AA36" s="2"/>
-      <c r="AB36" s="33"/>
-      <c r="AC36" s="33"/>
+      <c r="AB36" s="19"/>
+      <c r="AC36" s="19"/>
     </row>
     <row r="37" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="21"/>
+      <c r="A37" s="37"/>
       <c r="B37" s="4">
         <v>4</v>
       </c>
@@ -30760,11 +30817,11 @@
       <c r="Y37" s="2"/>
       <c r="Z37" s="2"/>
       <c r="AA37" s="2"/>
-      <c r="AB37" s="33"/>
-      <c r="AC37" s="33"/>
+      <c r="AB37" s="19"/>
+      <c r="AC37" s="19"/>
     </row>
     <row r="38" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="21"/>
+      <c r="A38" s="37"/>
       <c r="B38" s="4">
         <v>6</v>
       </c>
@@ -30799,11 +30856,11 @@
       <c r="Y38" s="2"/>
       <c r="Z38" s="2"/>
       <c r="AA38" s="2"/>
-      <c r="AB38" s="33"/>
-      <c r="AC38" s="33"/>
+      <c r="AB38" s="19"/>
+      <c r="AC38" s="19"/>
     </row>
     <row r="39" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="21"/>
+      <c r="A39" s="37"/>
       <c r="B39" s="4">
         <v>8</v>
       </c>
@@ -30838,11 +30895,11 @@
       <c r="Y39" s="2"/>
       <c r="Z39" s="2"/>
       <c r="AA39" s="2"/>
-      <c r="AB39" s="33"/>
-      <c r="AC39" s="33"/>
+      <c r="AB39" s="19"/>
+      <c r="AC39" s="19"/>
     </row>
     <row r="40" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="21"/>
+      <c r="A40" s="37"/>
       <c r="B40" s="4">
         <v>10</v>
       </c>
@@ -30877,11 +30934,11 @@
       <c r="Y40" s="2"/>
       <c r="Z40" s="2"/>
       <c r="AA40" s="2"/>
-      <c r="AB40" s="33"/>
-      <c r="AC40" s="33"/>
+      <c r="AB40" s="19"/>
+      <c r="AC40" s="19"/>
     </row>
     <row r="41" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="21"/>
+      <c r="A41" s="37"/>
       <c r="B41" s="4">
         <v>12</v>
       </c>
@@ -30916,11 +30973,11 @@
       <c r="Y41" s="2"/>
       <c r="Z41" s="2"/>
       <c r="AA41" s="2"/>
-      <c r="AB41" s="33"/>
-      <c r="AC41" s="33"/>
+      <c r="AB41" s="19"/>
+      <c r="AC41" s="19"/>
     </row>
     <row r="42" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="21"/>
+      <c r="A42" s="37"/>
       <c r="B42" s="4">
         <v>14</v>
       </c>
@@ -30955,11 +31012,11 @@
       <c r="Y42" s="2"/>
       <c r="Z42" s="2"/>
       <c r="AA42" s="2"/>
-      <c r="AB42" s="33"/>
-      <c r="AC42" s="33"/>
+      <c r="AB42" s="19"/>
+      <c r="AC42" s="19"/>
     </row>
     <row r="43" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="21"/>
+      <c r="A43" s="37"/>
       <c r="B43" s="4">
         <v>16</v>
       </c>
@@ -30994,11 +31051,11 @@
       <c r="Y43" s="2"/>
       <c r="Z43" s="2"/>
       <c r="AA43" s="2"/>
-      <c r="AB43" s="33"/>
-      <c r="AC43" s="33"/>
+      <c r="AB43" s="19"/>
+      <c r="AC43" s="19"/>
     </row>
     <row r="44" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="21"/>
+      <c r="A44" s="37"/>
       <c r="B44" s="4">
         <v>18</v>
       </c>
@@ -31033,11 +31090,11 @@
       <c r="Y44" s="2"/>
       <c r="Z44" s="2"/>
       <c r="AA44" s="2"/>
-      <c r="AB44" s="33"/>
-      <c r="AC44" s="33"/>
+      <c r="AB44" s="19"/>
+      <c r="AC44" s="19"/>
     </row>
     <row r="45" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="21"/>
+      <c r="A45" s="37"/>
       <c r="B45" s="4">
         <v>20</v>
       </c>
@@ -31072,11 +31129,11 @@
       <c r="Y45" s="2"/>
       <c r="Z45" s="2"/>
       <c r="AA45" s="2"/>
-      <c r="AB45" s="33"/>
-      <c r="AC45" s="33"/>
+      <c r="AB45" s="19"/>
+      <c r="AC45" s="19"/>
     </row>
     <row r="46" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="21"/>
+      <c r="A46" s="37"/>
       <c r="B46" s="10">
         <v>40</v>
       </c>
@@ -31111,17 +31168,17 @@
       <c r="Y46" s="2"/>
       <c r="Z46" s="2"/>
       <c r="AA46" s="2"/>
-      <c r="AB46" s="33"/>
-      <c r="AC46" s="33"/>
+      <c r="AB46" s="19"/>
+      <c r="AC46" s="19"/>
     </row>
     <row r="47" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="21"/>
-      <c r="B47" s="29" t="s">
+      <c r="A47" s="37"/>
+      <c r="B47" s="38" t="s">
         <v>8</v>
       </c>
-      <c r="C47" s="29"/>
-      <c r="D47" s="29"/>
-      <c r="E47" s="29"/>
+      <c r="C47" s="38"/>
+      <c r="D47" s="38"/>
+      <c r="E47" s="38"/>
       <c r="F47" s="2"/>
       <c r="G47" s="2"/>
       <c r="H47" s="2"/>
@@ -31144,11 +31201,11 @@
       <c r="Y47" s="2"/>
       <c r="Z47" s="2"/>
       <c r="AA47" s="2"/>
-      <c r="AB47" s="33"/>
-      <c r="AC47" s="33"/>
+      <c r="AB47" s="19"/>
+      <c r="AC47" s="19"/>
     </row>
     <row r="48" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="21"/>
+      <c r="A48" s="37"/>
       <c r="B48" s="3" t="s">
         <v>4</v>
       </c>
@@ -31183,11 +31240,11 @@
       <c r="Y48" s="8"/>
       <c r="Z48" s="8"/>
       <c r="AA48" s="8"/>
-      <c r="AB48" s="34"/>
-      <c r="AC48" s="34"/>
+      <c r="AB48" s="20"/>
+      <c r="AC48" s="20"/>
     </row>
     <row r="49" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="21"/>
+      <c r="A49" s="37"/>
       <c r="B49" s="4">
         <v>1</v>
       </c>
@@ -31225,11 +31282,11 @@
       <c r="Y49" s="8"/>
       <c r="Z49" s="8"/>
       <c r="AA49" s="8"/>
-      <c r="AB49" s="34"/>
-      <c r="AC49" s="34"/>
+      <c r="AB49" s="20"/>
+      <c r="AC49" s="20"/>
     </row>
     <row r="50" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="21"/>
+      <c r="A50" s="37"/>
       <c r="B50" s="4">
         <v>2</v>
       </c>
@@ -31267,11 +31324,11 @@
       <c r="Y50" s="8"/>
       <c r="Z50" s="8"/>
       <c r="AA50" s="8"/>
-      <c r="AB50" s="34"/>
-      <c r="AC50" s="34"/>
+      <c r="AB50" s="20"/>
+      <c r="AC50" s="20"/>
     </row>
     <row r="51" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="21"/>
+      <c r="A51" s="37"/>
       <c r="B51" s="4">
         <v>4</v>
       </c>
@@ -31309,11 +31366,11 @@
       <c r="Y51" s="8"/>
       <c r="Z51" s="8"/>
       <c r="AA51" s="8"/>
-      <c r="AB51" s="34"/>
-      <c r="AC51" s="34"/>
+      <c r="AB51" s="20"/>
+      <c r="AC51" s="20"/>
     </row>
     <row r="52" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="21"/>
+      <c r="A52" s="37"/>
       <c r="B52" s="4">
         <v>6</v>
       </c>
@@ -31351,11 +31408,11 @@
       <c r="Y52" s="8"/>
       <c r="Z52" s="8"/>
       <c r="AA52" s="8"/>
-      <c r="AB52" s="34"/>
-      <c r="AC52" s="34"/>
+      <c r="AB52" s="20"/>
+      <c r="AC52" s="20"/>
     </row>
     <row r="53" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="21"/>
+      <c r="A53" s="37"/>
       <c r="B53" s="13">
         <v>8</v>
       </c>
@@ -31393,11 +31450,11 @@
       <c r="Y53" s="8"/>
       <c r="Z53" s="8"/>
       <c r="AA53" s="8"/>
-      <c r="AB53" s="34"/>
-      <c r="AC53" s="34"/>
+      <c r="AB53" s="20"/>
+      <c r="AC53" s="20"/>
     </row>
     <row r="54" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="21"/>
+      <c r="A54" s="37"/>
       <c r="B54" s="4">
         <v>10</v>
       </c>
@@ -31435,11 +31492,11 @@
       <c r="Y54" s="8"/>
       <c r="Z54" s="8"/>
       <c r="AA54" s="8"/>
-      <c r="AB54" s="34"/>
-      <c r="AC54" s="34"/>
+      <c r="AB54" s="20"/>
+      <c r="AC54" s="20"/>
     </row>
     <row r="55" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="21"/>
+      <c r="A55" s="37"/>
       <c r="B55" s="4">
         <v>12</v>
       </c>
@@ -31477,11 +31534,11 @@
       <c r="Y55" s="8"/>
       <c r="Z55" s="8"/>
       <c r="AA55" s="8"/>
-      <c r="AB55" s="34"/>
-      <c r="AC55" s="34"/>
+      <c r="AB55" s="20"/>
+      <c r="AC55" s="20"/>
     </row>
     <row r="56" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="21"/>
+      <c r="A56" s="37"/>
       <c r="B56" s="4">
         <v>14</v>
       </c>
@@ -31519,11 +31576,11 @@
       <c r="Y56" s="8"/>
       <c r="Z56" s="8"/>
       <c r="AA56" s="8"/>
-      <c r="AB56" s="34"/>
-      <c r="AC56" s="34"/>
+      <c r="AB56" s="20"/>
+      <c r="AC56" s="20"/>
     </row>
     <row r="57" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A57" s="21"/>
+      <c r="A57" s="37"/>
       <c r="B57" s="4">
         <v>16</v>
       </c>
@@ -31561,11 +31618,11 @@
       <c r="Y57" s="2"/>
       <c r="Z57" s="2"/>
       <c r="AA57" s="2"/>
-      <c r="AB57" s="33"/>
-      <c r="AC57" s="33"/>
+      <c r="AB57" s="19"/>
+      <c r="AC57" s="19"/>
     </row>
     <row r="58" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="21"/>
+      <c r="A58" s="37"/>
       <c r="B58" s="4">
         <v>18</v>
       </c>
@@ -31603,11 +31660,11 @@
       <c r="Y58" s="8"/>
       <c r="Z58" s="8"/>
       <c r="AA58" s="8"/>
-      <c r="AB58" s="34"/>
-      <c r="AC58" s="34"/>
+      <c r="AB58" s="20"/>
+      <c r="AC58" s="20"/>
     </row>
     <row r="59" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A59" s="21"/>
+      <c r="A59" s="37"/>
       <c r="B59" s="4">
         <v>20</v>
       </c>
@@ -31645,11 +31702,11 @@
       <c r="Y59" s="8"/>
       <c r="Z59" s="8"/>
       <c r="AA59" s="8"/>
-      <c r="AB59" s="34"/>
-      <c r="AC59" s="34"/>
+      <c r="AB59" s="20"/>
+      <c r="AC59" s="20"/>
     </row>
     <row r="60" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A60" s="21"/>
+      <c r="A60" s="37"/>
       <c r="B60" s="10">
         <v>40</v>
       </c>
@@ -31687,17 +31744,17 @@
       <c r="Y60" s="8"/>
       <c r="Z60" s="8"/>
       <c r="AA60" s="8"/>
-      <c r="AB60" s="34"/>
-      <c r="AC60" s="34"/>
+      <c r="AB60" s="20"/>
+      <c r="AC60" s="20"/>
     </row>
     <row r="61" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="21"/>
-      <c r="B61" s="29" t="s">
+      <c r="A61" s="37"/>
+      <c r="B61" s="38" t="s">
         <v>9</v>
       </c>
-      <c r="C61" s="29"/>
-      <c r="D61" s="29"/>
-      <c r="E61" s="29"/>
+      <c r="C61" s="38"/>
+      <c r="D61" s="38"/>
+      <c r="E61" s="38"/>
       <c r="F61" s="8"/>
       <c r="G61" s="8"/>
       <c r="H61" s="8"/>
@@ -31720,11 +31777,11 @@
       <c r="Y61" s="8"/>
       <c r="Z61" s="8"/>
       <c r="AA61" s="8"/>
-      <c r="AB61" s="34"/>
-      <c r="AC61" s="34"/>
+      <c r="AB61" s="20"/>
+      <c r="AC61" s="20"/>
     </row>
     <row r="62" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A62" s="21"/>
+      <c r="A62" s="37"/>
       <c r="B62" s="3" t="s">
         <v>4</v>
       </c>
@@ -31759,11 +31816,11 @@
       <c r="Y62" s="8"/>
       <c r="Z62" s="8"/>
       <c r="AA62" s="8"/>
-      <c r="AB62" s="34"/>
-      <c r="AC62" s="34"/>
+      <c r="AB62" s="20"/>
+      <c r="AC62" s="20"/>
     </row>
     <row r="63" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A63" s="21"/>
+      <c r="A63" s="37"/>
       <c r="B63" s="4">
         <v>1</v>
       </c>
@@ -31801,11 +31858,11 @@
       <c r="Y63" s="8"/>
       <c r="Z63" s="8"/>
       <c r="AA63" s="8"/>
-      <c r="AB63" s="34"/>
-      <c r="AC63" s="34"/>
+      <c r="AB63" s="20"/>
+      <c r="AC63" s="20"/>
     </row>
     <row r="64" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="21"/>
+      <c r="A64" s="37"/>
       <c r="B64" s="4">
         <v>2</v>
       </c>
@@ -31843,11 +31900,11 @@
       <c r="Y64" s="8"/>
       <c r="Z64" s="8"/>
       <c r="AA64" s="8"/>
-      <c r="AB64" s="34"/>
-      <c r="AC64" s="34"/>
+      <c r="AB64" s="20"/>
+      <c r="AC64" s="20"/>
     </row>
     <row r="65" spans="1:30" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A65" s="21"/>
+      <c r="A65" s="37"/>
       <c r="B65" s="4">
         <v>4</v>
       </c>
@@ -31885,11 +31942,11 @@
       <c r="Y65" s="8"/>
       <c r="Z65" s="8"/>
       <c r="AA65" s="8"/>
-      <c r="AB65" s="34"/>
-      <c r="AC65" s="34"/>
+      <c r="AB65" s="20"/>
+      <c r="AC65" s="20"/>
     </row>
     <row r="66" spans="1:30" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A66" s="21"/>
+      <c r="A66" s="37"/>
       <c r="B66" s="4">
         <v>6</v>
       </c>
@@ -31927,11 +31984,11 @@
       <c r="Y66" s="8"/>
       <c r="Z66" s="8"/>
       <c r="AA66" s="8"/>
-      <c r="AB66" s="34"/>
-      <c r="AC66" s="34"/>
+      <c r="AB66" s="20"/>
+      <c r="AC66" s="20"/>
     </row>
     <row r="67" spans="1:30" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A67" s="21"/>
+      <c r="A67" s="37"/>
       <c r="B67" s="15">
         <v>8</v>
       </c>
@@ -31969,11 +32026,11 @@
       <c r="Y67" s="8"/>
       <c r="Z67" s="8"/>
       <c r="AA67" s="8"/>
-      <c r="AB67" s="34"/>
-      <c r="AC67" s="34"/>
+      <c r="AB67" s="20"/>
+      <c r="AC67" s="20"/>
     </row>
     <row r="68" spans="1:30" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A68" s="21"/>
+      <c r="A68" s="37"/>
       <c r="B68" s="4">
         <v>10</v>
       </c>
@@ -32011,11 +32068,11 @@
       <c r="Y68" s="8"/>
       <c r="Z68" s="8"/>
       <c r="AA68" s="8"/>
-      <c r="AB68" s="34"/>
-      <c r="AC68" s="34"/>
+      <c r="AB68" s="20"/>
+      <c r="AC68" s="20"/>
     </row>
     <row r="69" spans="1:30" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A69" s="21"/>
+      <c r="A69" s="37"/>
       <c r="B69" s="4">
         <v>12</v>
       </c>
@@ -32053,11 +32110,11 @@
       <c r="Y69" s="2"/>
       <c r="Z69" s="2"/>
       <c r="AA69" s="2"/>
-      <c r="AB69" s="33"/>
-      <c r="AC69" s="33"/>
+      <c r="AB69" s="19"/>
+      <c r="AC69" s="19"/>
     </row>
     <row r="70" spans="1:30" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A70" s="21"/>
+      <c r="A70" s="37"/>
       <c r="B70" s="4">
         <v>14</v>
       </c>
@@ -32095,11 +32152,11 @@
       <c r="Y70" s="2"/>
       <c r="Z70" s="2"/>
       <c r="AA70" s="2"/>
-      <c r="AB70" s="33"/>
-      <c r="AC70" s="33"/>
+      <c r="AB70" s="19"/>
+      <c r="AC70" s="19"/>
     </row>
     <row r="71" spans="1:30" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A71" s="21"/>
+      <c r="A71" s="37"/>
       <c r="B71" s="4">
         <v>16</v>
       </c>
@@ -32137,11 +32194,11 @@
       <c r="Y71" s="8"/>
       <c r="Z71" s="8"/>
       <c r="AA71" s="8"/>
-      <c r="AB71" s="34"/>
-      <c r="AC71" s="34"/>
+      <c r="AB71" s="20"/>
+      <c r="AC71" s="20"/>
     </row>
     <row r="72" spans="1:30" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A72" s="21"/>
+      <c r="A72" s="37"/>
       <c r="B72" s="4">
         <v>18</v>
       </c>
@@ -32179,12 +32236,12 @@
       <c r="Y72" s="8"/>
       <c r="Z72" s="8"/>
       <c r="AA72" s="8"/>
-      <c r="AB72" s="35"/>
-      <c r="AC72" s="35"/>
-      <c r="AD72" s="36"/>
+      <c r="AB72" s="21"/>
+      <c r="AC72" s="21"/>
+      <c r="AD72" s="22"/>
     </row>
     <row r="73" spans="1:30" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A73" s="21"/>
+      <c r="A73" s="37"/>
       <c r="B73" s="4">
         <v>20</v>
       </c>
@@ -32222,12 +32279,12 @@
       <c r="Y73" s="8"/>
       <c r="Z73" s="8"/>
       <c r="AA73" s="8"/>
-      <c r="AB73" s="35"/>
-      <c r="AC73" s="35"/>
-      <c r="AD73" s="36"/>
+      <c r="AB73" s="21"/>
+      <c r="AC73" s="21"/>
+      <c r="AD73" s="22"/>
     </row>
     <row r="74" spans="1:30" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A74" s="21"/>
+      <c r="A74" s="37"/>
       <c r="B74" s="10">
         <v>40</v>
       </c>
@@ -32265,56 +32322,56 @@
       <c r="Y74" s="8"/>
       <c r="Z74" s="8"/>
       <c r="AA74" s="8"/>
-      <c r="AB74" s="35"/>
-      <c r="AC74" s="35"/>
-      <c r="AD74" s="36"/>
+      <c r="AB74" s="21"/>
+      <c r="AC74" s="21"/>
+      <c r="AD74" s="22"/>
     </row>
     <row r="75" spans="1:30" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A75" s="21"/>
+      <c r="A75" s="37"/>
       <c r="B75" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="C75" s="39" t="s">
+      <c r="C75" s="41" t="s">
         <v>14</v>
       </c>
-      <c r="D75" s="39"/>
-      <c r="E75" s="39"/>
-      <c r="F75" s="39"/>
-      <c r="G75" s="39"/>
-      <c r="H75" s="39"/>
-      <c r="I75" s="39"/>
-      <c r="J75" s="39"/>
-      <c r="K75" s="39"/>
-      <c r="L75" s="39"/>
-      <c r="M75" s="39"/>
-      <c r="N75" s="39"/>
-      <c r="O75" s="39"/>
-      <c r="P75" s="39"/>
-      <c r="Q75" s="39"/>
-      <c r="R75" s="39"/>
-      <c r="S75" s="39"/>
-      <c r="T75" s="39"/>
-      <c r="U75" s="39"/>
-      <c r="V75" s="39"/>
-      <c r="W75" s="39"/>
-      <c r="X75" s="39"/>
-      <c r="Y75" s="39"/>
-      <c r="Z75" s="39"/>
-      <c r="AA75" s="39"/>
-      <c r="AB75" s="37"/>
-      <c r="AC75" s="37"/>
-      <c r="AD75" s="36"/>
+      <c r="D75" s="41"/>
+      <c r="E75" s="41"/>
+      <c r="F75" s="41"/>
+      <c r="G75" s="41"/>
+      <c r="H75" s="41"/>
+      <c r="I75" s="41"/>
+      <c r="J75" s="41"/>
+      <c r="K75" s="41"/>
+      <c r="L75" s="41"/>
+      <c r="M75" s="41"/>
+      <c r="N75" s="41"/>
+      <c r="O75" s="41"/>
+      <c r="P75" s="41"/>
+      <c r="Q75" s="41"/>
+      <c r="R75" s="41"/>
+      <c r="S75" s="41"/>
+      <c r="T75" s="41"/>
+      <c r="U75" s="41"/>
+      <c r="V75" s="41"/>
+      <c r="W75" s="41"/>
+      <c r="X75" s="41"/>
+      <c r="Y75" s="41"/>
+      <c r="Z75" s="41"/>
+      <c r="AA75" s="41"/>
+      <c r="AB75" s="23"/>
+      <c r="AC75" s="23"/>
+      <c r="AD75" s="22"/>
     </row>
     <row r="76" spans="1:30" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A76" s="28" t="s">
+      <c r="A76" s="39" t="s">
         <v>15</v>
       </c>
-      <c r="B76" s="29" t="s">
+      <c r="B76" s="38" t="s">
         <v>3</v>
       </c>
-      <c r="C76" s="29"/>
-      <c r="D76" s="29"/>
-      <c r="E76" s="29"/>
+      <c r="C76" s="38"/>
+      <c r="D76" s="38"/>
+      <c r="E76" s="38"/>
       <c r="F76" s="2"/>
       <c r="G76" s="2"/>
       <c r="H76" s="2"/>
@@ -32337,12 +32394,12 @@
       <c r="Y76" s="1"/>
       <c r="Z76" s="1"/>
       <c r="AA76" s="1"/>
-      <c r="AB76" s="38"/>
-      <c r="AC76" s="38"/>
-      <c r="AD76" s="36"/>
+      <c r="AB76" s="24"/>
+      <c r="AC76" s="24"/>
+      <c r="AD76" s="22"/>
     </row>
     <row r="77" spans="1:30" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A77" s="28"/>
+      <c r="A77" s="39"/>
       <c r="B77" s="3" t="s">
         <v>4</v>
       </c>
@@ -32377,12 +32434,12 @@
       <c r="Y77" s="1"/>
       <c r="Z77" s="1"/>
       <c r="AA77" s="1"/>
-      <c r="AB77" s="38"/>
-      <c r="AC77" s="38"/>
-      <c r="AD77" s="36"/>
+      <c r="AB77" s="24"/>
+      <c r="AC77" s="24"/>
+      <c r="AD77" s="22"/>
     </row>
     <row r="78" spans="1:30" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A78" s="28"/>
+      <c r="A78" s="39"/>
       <c r="B78" s="4">
         <v>1</v>
       </c>
@@ -32417,12 +32474,12 @@
       <c r="Y78" s="1"/>
       <c r="Z78" s="1"/>
       <c r="AA78" s="1"/>
-      <c r="AB78" s="38"/>
-      <c r="AC78" s="38"/>
-      <c r="AD78" s="36"/>
+      <c r="AB78" s="24"/>
+      <c r="AC78" s="24"/>
+      <c r="AD78" s="22"/>
     </row>
     <row r="79" spans="1:30" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A79" s="28"/>
+      <c r="A79" s="39"/>
       <c r="B79" s="4">
         <v>2</v>
       </c>
@@ -32461,7 +32518,7 @@
       <c r="AC79" s="1"/>
     </row>
     <row r="80" spans="1:30" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A80" s="28"/>
+      <c r="A80" s="39"/>
       <c r="B80" s="4">
         <v>4</v>
       </c>
@@ -32500,7 +32557,7 @@
       <c r="AC80" s="1"/>
     </row>
     <row r="81" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A81" s="28"/>
+      <c r="A81" s="39"/>
       <c r="B81" s="4">
         <v>6</v>
       </c>
@@ -32539,7 +32596,7 @@
       <c r="AC81" s="1"/>
     </row>
     <row r="82" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A82" s="28"/>
+      <c r="A82" s="39"/>
       <c r="B82" s="4">
         <v>8</v>
       </c>
@@ -32578,13 +32635,13 @@
       <c r="AC82" s="1"/>
     </row>
     <row r="83" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A83" s="28"/>
-      <c r="B83" s="29" t="s">
+      <c r="A83" s="39"/>
+      <c r="B83" s="38" t="s">
         <v>8</v>
       </c>
-      <c r="C83" s="29"/>
-      <c r="D83" s="29"/>
-      <c r="E83" s="29"/>
+      <c r="C83" s="38"/>
+      <c r="D83" s="38"/>
+      <c r="E83" s="38"/>
       <c r="F83" s="2"/>
       <c r="G83" s="2"/>
       <c r="H83" s="2"/>
@@ -32611,7 +32668,7 @@
       <c r="AC83" s="1"/>
     </row>
     <row r="84" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A84" s="28"/>
+      <c r="A84" s="39"/>
       <c r="B84" s="3" t="s">
         <v>4</v>
       </c>
@@ -32650,7 +32707,7 @@
       <c r="AC84" s="1"/>
     </row>
     <row r="85" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A85" s="28"/>
+      <c r="A85" s="39"/>
       <c r="B85" s="3">
         <v>1</v>
       </c>
@@ -32692,7 +32749,7 @@
       <c r="AC85" s="1"/>
     </row>
     <row r="86" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A86" s="28"/>
+      <c r="A86" s="39"/>
       <c r="B86" s="3">
         <v>2</v>
       </c>
@@ -32734,7 +32791,7 @@
       <c r="AC86" s="1"/>
     </row>
     <row r="87" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A87" s="28"/>
+      <c r="A87" s="39"/>
       <c r="B87" s="3">
         <v>4</v>
       </c>
@@ -32776,7 +32833,7 @@
       <c r="AC87" s="1"/>
     </row>
     <row r="88" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A88" s="28"/>
+      <c r="A88" s="39"/>
       <c r="B88" s="3">
         <v>6</v>
       </c>
@@ -32818,7 +32875,7 @@
       <c r="AC88" s="1"/>
     </row>
     <row r="89" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A89" s="28"/>
+      <c r="A89" s="39"/>
       <c r="B89" s="17">
         <v>8</v>
       </c>
@@ -32860,13 +32917,13 @@
       <c r="AC89" s="1"/>
     </row>
     <row r="90" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A90" s="28"/>
-      <c r="B90" s="29" t="s">
+      <c r="A90" s="39"/>
+      <c r="B90" s="38" t="s">
         <v>9</v>
       </c>
-      <c r="C90" s="29"/>
-      <c r="D90" s="29"/>
-      <c r="E90" s="29"/>
+      <c r="C90" s="38"/>
+      <c r="D90" s="38"/>
+      <c r="E90" s="38"/>
       <c r="F90" s="7"/>
       <c r="G90" s="7"/>
       <c r="H90" s="8"/>
@@ -32893,7 +32950,7 @@
       <c r="AC90" s="1"/>
     </row>
     <row r="91" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A91" s="28"/>
+      <c r="A91" s="39"/>
       <c r="B91" s="3" t="s">
         <v>4</v>
       </c>
@@ -32932,7 +32989,7 @@
       <c r="AC91" s="1"/>
     </row>
     <row r="92" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A92" s="28"/>
+      <c r="A92" s="39"/>
       <c r="B92" s="3">
         <v>1</v>
       </c>
@@ -32974,7 +33031,7 @@
       <c r="AC92" s="1"/>
     </row>
     <row r="93" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A93" s="28"/>
+      <c r="A93" s="39"/>
       <c r="B93" s="3">
         <v>2</v>
       </c>
@@ -33016,7 +33073,7 @@
       <c r="AC93" s="1"/>
     </row>
     <row r="94" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A94" s="28"/>
+      <c r="A94" s="39"/>
       <c r="B94" s="3">
         <v>4</v>
       </c>
@@ -33058,7 +33115,7 @@
       <c r="AC94" s="1"/>
     </row>
     <row r="95" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A95" s="28"/>
+      <c r="A95" s="39"/>
       <c r="B95" s="3">
         <v>6</v>
       </c>
@@ -33100,7 +33157,7 @@
       <c r="AC95" s="1"/>
     </row>
     <row r="96" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A96" s="28"/>
+      <c r="A96" s="39"/>
       <c r="B96" s="18">
         <v>8</v>
       </c>
@@ -33142,13 +33199,13 @@
       <c r="AC96" s="1"/>
     </row>
     <row r="97" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A97" s="28"/>
-      <c r="B97" s="30" t="s">
+      <c r="A97" s="39"/>
+      <c r="B97" s="40" t="s">
         <v>10</v>
       </c>
-      <c r="C97" s="30"/>
-      <c r="D97" s="30"/>
-      <c r="E97" s="30"/>
+      <c r="C97" s="40"/>
+      <c r="D97" s="40"/>
+      <c r="E97" s="40"/>
       <c r="F97" s="7"/>
       <c r="G97" s="7"/>
       <c r="H97" s="8"/>
@@ -33175,13 +33232,13 @@
       <c r="AC97" s="1"/>
     </row>
     <row r="98" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A98" s="28"/>
-      <c r="B98" s="19" t="s">
+      <c r="A98" s="39"/>
+      <c r="B98" s="35" t="s">
         <v>17</v>
       </c>
-      <c r="C98" s="19"/>
-      <c r="D98" s="19"/>
-      <c r="E98" s="19"/>
+      <c r="C98" s="35"/>
+      <c r="D98" s="35"/>
+      <c r="E98" s="35"/>
       <c r="F98" s="7"/>
       <c r="G98" s="7"/>
       <c r="H98" s="8"/>
@@ -33208,11 +33265,11 @@
       <c r="AC98" s="1"/>
     </row>
     <row r="99" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A99" s="28"/>
-      <c r="B99" s="19"/>
-      <c r="C99" s="19"/>
-      <c r="D99" s="19"/>
-      <c r="E99" s="19"/>
+      <c r="A99" s="39"/>
+      <c r="B99" s="35"/>
+      <c r="C99" s="35"/>
+      <c r="D99" s="35"/>
+      <c r="E99" s="35"/>
       <c r="F99" s="7"/>
       <c r="G99" s="7"/>
       <c r="H99" s="8"/>
@@ -33239,11 +33296,11 @@
       <c r="AC99" s="1"/>
     </row>
     <row r="100" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A100" s="28"/>
-      <c r="B100" s="19"/>
-      <c r="C100" s="19"/>
-      <c r="D100" s="19"/>
-      <c r="E100" s="19"/>
+      <c r="A100" s="39"/>
+      <c r="B100" s="35"/>
+      <c r="C100" s="35"/>
+      <c r="D100" s="35"/>
+      <c r="E100" s="35"/>
       <c r="F100" s="7"/>
       <c r="G100" s="7"/>
       <c r="H100" s="8"/>
@@ -33270,11 +33327,11 @@
       <c r="AC100" s="1"/>
     </row>
     <row r="101" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A101" s="28"/>
-      <c r="B101" s="19"/>
-      <c r="C101" s="19"/>
-      <c r="D101" s="19"/>
-      <c r="E101" s="19"/>
+      <c r="A101" s="39"/>
+      <c r="B101" s="35"/>
+      <c r="C101" s="35"/>
+      <c r="D101" s="35"/>
+      <c r="E101" s="35"/>
       <c r="F101" s="7"/>
       <c r="G101" s="7"/>
       <c r="H101" s="8"/>
@@ -33301,11 +33358,11 @@
       <c r="AC101" s="1"/>
     </row>
     <row r="102" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A102" s="28"/>
-      <c r="B102" s="19"/>
-      <c r="C102" s="19"/>
-      <c r="D102" s="19"/>
-      <c r="E102" s="19"/>
+      <c r="A102" s="39"/>
+      <c r="B102" s="35"/>
+      <c r="C102" s="35"/>
+      <c r="D102" s="35"/>
+      <c r="E102" s="35"/>
       <c r="F102" s="7"/>
       <c r="G102" s="7"/>
       <c r="H102" s="8"/>
@@ -33332,11 +33389,11 @@
       <c r="AC102" s="1"/>
     </row>
     <row r="103" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A103" s="28"/>
-      <c r="B103" s="19"/>
-      <c r="C103" s="19"/>
-      <c r="D103" s="19"/>
-      <c r="E103" s="19"/>
+      <c r="A103" s="39"/>
+      <c r="B103" s="35"/>
+      <c r="C103" s="35"/>
+      <c r="D103" s="35"/>
+      <c r="E103" s="35"/>
       <c r="F103" s="7"/>
       <c r="G103" s="7"/>
       <c r="H103" s="8"/>
@@ -33363,11 +33420,11 @@
       <c r="AC103" s="1"/>
     </row>
     <row r="104" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A104" s="28"/>
-      <c r="B104" s="19"/>
-      <c r="C104" s="19"/>
-      <c r="D104" s="19"/>
-      <c r="E104" s="19"/>
+      <c r="A104" s="39"/>
+      <c r="B104" s="35"/>
+      <c r="C104" s="35"/>
+      <c r="D104" s="35"/>
+      <c r="E104" s="35"/>
       <c r="F104" s="2"/>
       <c r="G104" s="2"/>
       <c r="H104" s="2"/>
@@ -33394,11 +33451,11 @@
       <c r="AC104" s="1"/>
     </row>
     <row r="105" spans="1:29" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A105" s="28"/>
-      <c r="B105" s="19"/>
-      <c r="C105" s="19"/>
-      <c r="D105" s="19"/>
-      <c r="E105" s="19"/>
+      <c r="A105" s="39"/>
+      <c r="B105" s="35"/>
+      <c r="C105" s="35"/>
+      <c r="D105" s="35"/>
+      <c r="E105" s="35"/>
       <c r="F105" s="2"/>
       <c r="G105" s="2"/>
       <c r="H105" s="2"/>
@@ -33457,270 +33514,402 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{20DD6B2D-C446-466B-9C71-121C80824D6F}">
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:L26"/>
   <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="66.7109375" bestFit="1" customWidth="1"/>
     <col min="2" max="5" width="21.7109375" customWidth="1"/>
+    <col min="7" max="11" width="11.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="17.3" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="31" t="s">
+    <row r="1" spans="1:12" ht="17.3" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="42" t="s">
         <v>18</v>
       </c>
-      <c r="B1" s="32"/>
-      <c r="C1" s="40"/>
-      <c r="D1" s="49" t="s">
+      <c r="B1" s="43"/>
+      <c r="C1" s="59"/>
+      <c r="D1" s="60" t="s">
         <v>19</v>
       </c>
-      <c r="E1" s="49" t="s">
+      <c r="E1" s="60" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="17.3" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="41" t="s">
+    <row r="2" spans="1:12" ht="17.3" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="25" t="s">
         <v>21</v>
       </c>
-      <c r="B2" s="42" t="s">
+      <c r="B2" s="61" t="s">
         <v>22</v>
       </c>
-      <c r="C2" s="42"/>
-      <c r="D2" s="42"/>
-      <c r="E2" s="42"/>
+      <c r="C2" s="61"/>
+      <c r="D2" s="61"/>
+      <c r="E2" s="61"/>
     </row>
-    <row r="3" spans="1:5" ht="17.3" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="43" t="s">
+    <row r="3" spans="1:12" ht="17.3" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="58" t="s">
         <v>23</v>
       </c>
-      <c r="B3" s="43"/>
-      <c r="C3" s="43"/>
-      <c r="D3" s="43"/>
-      <c r="E3" s="43"/>
+      <c r="B3" s="58"/>
+      <c r="C3" s="58"/>
+      <c r="D3" s="58"/>
+      <c r="E3" s="58"/>
     </row>
-    <row r="4" spans="1:5" ht="17.3" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="44" t="s">
+    <row r="4" spans="1:12" ht="17.3" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="26" t="s">
         <v>24</v>
       </c>
-      <c r="B4" s="45">
+      <c r="B4" s="27">
         <v>1000</v>
       </c>
-      <c r="C4" s="45">
+      <c r="C4" s="27">
         <v>3000</v>
       </c>
-      <c r="D4" s="45">
+      <c r="D4" s="27">
         <v>7000</v>
       </c>
-      <c r="E4" s="45">
+      <c r="E4" s="27">
         <v>10000</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="17.3" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="44" t="s">
+    <row r="5" spans="1:12" ht="17.3" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="26" t="s">
         <v>25</v>
       </c>
-      <c r="B5" s="46">
+      <c r="B5" s="28">
         <v>13</v>
       </c>
-      <c r="C5" s="46">
+      <c r="C5" s="28">
         <v>117</v>
       </c>
-      <c r="D5" s="46">
+      <c r="D5" s="28">
         <v>633</v>
       </c>
-      <c r="E5" s="46">
+      <c r="E5" s="28">
         <v>1101</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="17.3" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="47" t="s">
+    <row r="6" spans="1:12" ht="17.3" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="29" t="s">
         <v>26</v>
       </c>
-      <c r="B6" s="48">
+      <c r="B6" s="30">
         <v>50</v>
       </c>
-      <c r="C6" s="48">
+      <c r="C6" s="30">
         <v>461</v>
       </c>
-      <c r="D6" s="48">
+      <c r="D6" s="30">
         <v>4644</v>
       </c>
-      <c r="E6" s="48">
+      <c r="E6" s="30">
         <v>11709</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="17.3" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="44" t="s">
+    <row r="7" spans="1:12" ht="17.3" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="26" t="s">
         <v>27</v>
       </c>
-      <c r="B7" s="46">
+      <c r="B7" s="28">
         <v>64</v>
       </c>
-      <c r="C7" s="46">
+      <c r="C7" s="28">
         <v>582</v>
       </c>
-      <c r="D7" s="46">
+      <c r="D7" s="28">
         <v>5284</v>
       </c>
-      <c r="E7" s="46">
+      <c r="E7" s="28">
         <v>12810</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="17.3" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="43" t="s">
+    <row r="8" spans="1:12" ht="17.3" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="58" t="s">
         <v>28</v>
       </c>
-      <c r="B8" s="43"/>
-      <c r="C8" s="43"/>
-      <c r="D8" s="43"/>
-      <c r="E8" s="43"/>
+      <c r="B8" s="58"/>
+      <c r="C8" s="58"/>
+      <c r="D8" s="58"/>
+      <c r="E8" s="58"/>
+      <c r="F8" s="31"/>
+      <c r="G8" s="31"/>
+      <c r="H8" s="31"/>
+      <c r="I8" s="31"/>
+      <c r="J8" s="31"/>
+      <c r="K8" s="31"/>
+      <c r="L8" s="31"/>
     </row>
-    <row r="9" spans="1:5" ht="17.3" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="44" t="s">
+    <row r="9" spans="1:12" ht="17.3" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="26" t="s">
         <v>24</v>
       </c>
-      <c r="B9" s="45">
+      <c r="B9" s="27">
         <v>3000</v>
       </c>
-      <c r="C9" s="45">
+      <c r="C9" s="27">
         <v>5000</v>
       </c>
-      <c r="D9" s="45">
+      <c r="D9" s="27">
         <v>7000</v>
       </c>
-      <c r="E9" s="45">
+      <c r="E9" s="27">
         <v>10000</v>
       </c>
+      <c r="F9" s="31"/>
+      <c r="G9" s="31"/>
+      <c r="H9" s="31"/>
+      <c r="I9" s="31"/>
+      <c r="J9" s="31"/>
+      <c r="K9" s="31"/>
+      <c r="L9" s="31"/>
     </row>
-    <row r="10" spans="1:5" ht="17.3" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="44" t="s">
+    <row r="10" spans="1:12" ht="17.3" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="26" t="s">
         <v>25</v>
       </c>
-      <c r="B10" s="46">
+      <c r="B10" s="28">
         <v>1175</v>
       </c>
-      <c r="C10" s="46">
+      <c r="C10" s="28">
         <v>2668</v>
       </c>
-      <c r="D10" s="46">
+      <c r="D10" s="28">
         <v>4787</v>
       </c>
-      <c r="E10" s="46">
+      <c r="E10" s="28">
         <v>9358</v>
       </c>
+      <c r="F10" s="31"/>
+      <c r="G10" s="31"/>
+      <c r="H10" s="31"/>
+      <c r="I10" s="31"/>
+      <c r="J10" s="31"/>
+      <c r="K10" s="31"/>
+      <c r="L10" s="31"/>
     </row>
-    <row r="11" spans="1:5" ht="17.3" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="47" t="s">
+    <row r="11" spans="1:12" ht="17.3" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="29" t="s">
         <v>26</v>
       </c>
-      <c r="B11" s="48">
+      <c r="B11" s="30">
         <v>514</v>
       </c>
-      <c r="C11" s="48">
+      <c r="C11" s="30">
         <v>719</v>
       </c>
-      <c r="D11" s="48">
+      <c r="D11" s="30">
         <v>1689</v>
       </c>
-      <c r="E11" s="48">
+      <c r="E11" s="30">
         <v>3658</v>
       </c>
+      <c r="F11" s="31"/>
+      <c r="G11" s="31"/>
+      <c r="H11" s="31"/>
+      <c r="I11" s="31"/>
+      <c r="J11" s="31"/>
+      <c r="K11" s="31"/>
+      <c r="L11" s="31"/>
     </row>
-    <row r="12" spans="1:5" ht="17.3" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="44" t="s">
+    <row r="12" spans="1:12" ht="17.3" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="26" t="s">
         <v>27</v>
       </c>
-      <c r="B12" s="46">
+      <c r="B12" s="28">
         <v>1689</v>
       </c>
-      <c r="C12" s="46">
+      <c r="C12" s="28">
         <v>3387</v>
       </c>
-      <c r="D12" s="46">
+      <c r="D12" s="28">
         <v>6476</v>
       </c>
-      <c r="E12" s="46">
+      <c r="E12" s="28">
         <v>12974</v>
       </c>
+      <c r="F12" s="31"/>
+      <c r="G12" s="31"/>
+      <c r="H12" s="31"/>
+      <c r="I12" s="31"/>
+      <c r="J12" s="31"/>
+      <c r="K12" s="31"/>
+      <c r="L12" s="31"/>
     </row>
-    <row r="13" spans="1:5" ht="17.3" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="43" t="s">
+    <row r="13" spans="1:12" ht="17.3" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="58" t="s">
         <v>29</v>
       </c>
-      <c r="B13" s="43"/>
-      <c r="C13" s="43"/>
-      <c r="D13" s="43"/>
-      <c r="E13" s="43"/>
+      <c r="B13" s="58"/>
+      <c r="C13" s="58"/>
+      <c r="D13" s="58"/>
+      <c r="E13" s="58"/>
+      <c r="F13" s="31"/>
+      <c r="L13" s="31"/>
     </row>
-    <row r="14" spans="1:5" ht="17.3" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="44" t="s">
+    <row r="14" spans="1:12" ht="17.3" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="26" t="s">
         <v>24</v>
       </c>
-      <c r="B14" s="45">
+      <c r="B14" s="27">
         <v>2000</v>
       </c>
-      <c r="C14" s="45">
+      <c r="C14" s="27">
         <v>3000</v>
       </c>
-      <c r="D14" s="45">
+      <c r="D14" s="27">
         <v>5000</v>
       </c>
-      <c r="E14" s="45">
+      <c r="E14" s="27">
         <v>7000</v>
       </c>
+      <c r="F14" s="31"/>
+      <c r="G14" s="56" t="s">
+        <v>31</v>
+      </c>
+      <c r="H14" s="53" t="s">
+        <v>30</v>
+      </c>
+      <c r="I14" s="54"/>
+      <c r="J14" s="54"/>
+      <c r="K14" s="55"/>
+      <c r="L14" s="31"/>
     </row>
-    <row r="15" spans="1:5" ht="17.3" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="44" t="s">
+    <row r="15" spans="1:12" ht="17.3" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="26" t="s">
         <v>25</v>
       </c>
-      <c r="B15" s="46">
-        <v>427</v>
-      </c>
-      <c r="C15" s="46">
-        <v>962</v>
-      </c>
-      <c r="D15" s="46">
-        <v>2591</v>
-      </c>
-      <c r="E15" s="46">
-        <v>5213</v>
-      </c>
+      <c r="B15" s="28"/>
+      <c r="C15" s="28"/>
+      <c r="D15" s="28"/>
+      <c r="E15" s="28"/>
+      <c r="F15" s="31"/>
+      <c r="G15" s="57"/>
+      <c r="H15" s="33">
+        <v>16</v>
+      </c>
+      <c r="I15" s="33">
+        <v>32</v>
+      </c>
+      <c r="J15" s="33">
+        <v>64</v>
+      </c>
+      <c r="K15" s="33">
+        <v>128</v>
+      </c>
+      <c r="L15" s="31"/>
     </row>
-    <row r="16" spans="1:5" ht="17.3" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="47" t="s">
+    <row r="16" spans="1:12" ht="17.3" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="29" t="s">
         <v>26</v>
       </c>
-      <c r="B16" s="48">
-        <v>1848</v>
-      </c>
-      <c r="C16" s="48">
-        <v>5601</v>
-      </c>
-      <c r="D16" s="48">
-        <v>24408</v>
-      </c>
-      <c r="E16" s="48">
-        <v>70536</v>
-      </c>
+      <c r="B16" s="30"/>
+      <c r="C16" s="30"/>
+      <c r="D16" s="30"/>
+      <c r="E16" s="30"/>
+      <c r="F16" s="31"/>
+      <c r="G16" s="33">
+        <v>2000</v>
+      </c>
+      <c r="H16" s="34">
+        <v>2256</v>
+      </c>
+      <c r="I16" s="34">
+        <v>1332</v>
+      </c>
+      <c r="J16" s="34">
+        <v>1844</v>
+      </c>
+      <c r="K16" s="34">
+        <v>4329</v>
+      </c>
+      <c r="L16" s="31"/>
     </row>
-    <row r="17" spans="1:5" ht="17.3" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="44" t="s">
+    <row r="17" spans="1:12" ht="17.3" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="26" t="s">
         <v>27</v>
       </c>
-      <c r="B17" s="46">
-        <v>2276</v>
-      </c>
-      <c r="C17" s="46">
-        <v>6563</v>
-      </c>
-      <c r="D17" s="46">
-        <v>26999</v>
-      </c>
-      <c r="E17" s="46">
-        <v>75750</v>
-      </c>
+      <c r="B17" s="28"/>
+      <c r="C17" s="28"/>
+      <c r="D17" s="28"/>
+      <c r="E17" s="28"/>
+      <c r="F17" s="31"/>
+      <c r="G17" s="33">
+        <v>3000</v>
+      </c>
+      <c r="H17" s="34">
+        <v>7481</v>
+      </c>
+      <c r="I17" s="34">
+        <v>4620</v>
+      </c>
+      <c r="J17" s="34">
+        <v>5585</v>
+      </c>
+      <c r="K17" s="34">
+        <v>13227</v>
+      </c>
+      <c r="L17" s="31"/>
+    </row>
+    <row r="18" spans="1:12" ht="17.850000000000001" x14ac:dyDescent="0.25">
+      <c r="F18" s="31"/>
+      <c r="L18" s="31"/>
+    </row>
+    <row r="19" spans="1:12" ht="17.850000000000001" x14ac:dyDescent="0.25">
+      <c r="F19" s="31"/>
+      <c r="G19" s="31"/>
+      <c r="H19" s="31"/>
+      <c r="I19" s="31"/>
+      <c r="J19" s="31"/>
+      <c r="K19" s="31"/>
+      <c r="L19" s="31"/>
+    </row>
+    <row r="20" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F20" s="31"/>
+      <c r="L20" s="31"/>
+    </row>
+    <row r="21" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F21" s="31"/>
+      <c r="L21" s="31"/>
+    </row>
+    <row r="22" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F22" s="31"/>
+      <c r="L22" s="31"/>
+    </row>
+    <row r="23" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F23" s="31"/>
+      <c r="L23" s="31"/>
+    </row>
+    <row r="24" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F24" s="20"/>
+      <c r="G24" s="32"/>
+      <c r="H24" s="32"/>
+      <c r="I24" s="32"/>
+      <c r="J24" s="32"/>
+      <c r="K24" s="32"/>
+      <c r="L24" s="20"/>
+    </row>
+    <row r="25" spans="1:12" ht="20" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F25" s="20"/>
+      <c r="G25" s="32"/>
+      <c r="H25" s="32"/>
+      <c r="I25" s="32"/>
+      <c r="J25" s="32"/>
+      <c r="K25" s="32"/>
+      <c r="L25" s="20"/>
+    </row>
+    <row r="26" spans="1:12" ht="17.850000000000001" x14ac:dyDescent="0.25">
+      <c r="F26" s="31"/>
+      <c r="G26" s="31"/>
+      <c r="H26" s="31"/>
+      <c r="I26" s="31"/>
+      <c r="J26" s="31"/>
+      <c r="K26" s="31"/>
+      <c r="L26" s="31"/>
     </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="8">
+    <mergeCell ref="H14:K14"/>
+    <mergeCell ref="G14:G15"/>
     <mergeCell ref="A13:E13"/>
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="D1:E1"/>
@@ -33733,6 +33922,7 @@
     <hyperlink ref="D1:E1" location="Графики!A1" display="Соотв. Графики" xr:uid="{1CAB3C67-9149-433C-ADF0-E6817A5FDD65}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>